<commit_message>
Add Date From / Date To columns to exception list
- Update exceptions.xlsx with Date From (col C) and Date To (col D)
- Add date parsing and range checking to load_exceptions()
- Permanent exclusion when both dates empty, bounded otherwise
- Skip rows with invalid dates gracefully

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/watchlists/exceptions.xlsx
+++ b/watchlists/exceptions.xlsx
@@ -422,11 +422,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -440,6 +442,16 @@
           <t>Reason</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Date From</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Date To</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -452,6 +464,8 @@
           <t>Too volatile - remove this row and add your own</t>
         </is>
       </c>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -464,6 +478,16 @@
           <t>Under regulatory review - replace with real tickers</t>
         </is>
       </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -476,6 +500,12 @@
           <t>Already holding this position - customize as needed</t>
         </is>
       </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Change exception list date format to dd/MMM/yyyy
- Update exceptions.xlsx examples to use dd/MMM/yyyy format
- Parse dates with strptime %d/%b/%Y in load_exceptions()
- Normalize month abbreviation to title-case for case-insensitive
  handling (jul, Jul, JUL all work)

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/watchlists/exceptions.xlsx
+++ b/watchlists/exceptions.xlsx
@@ -480,12 +480,12 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>01/Jan/2026</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-12-31</t>
+          <t>31/Dec/2026</t>
         </is>
       </c>
     </row>
@@ -502,7 +502,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>01/Jun/2026</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Stable release 2.0.0 - Top 20 ranking, exception list, cloud workflow
- Rank stocks by Market Cap, RSI, Strong Uptrend, Pullback to 20 MA
- Exception list (watchlists/exceptions.xlsx) with date range support
- GitHub Actions workflow for cloud scanning
- TOP_RESULTS set to 20
- Column order: Symbol, Date From, Date To, Reason

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/watchlists/exceptions.xlsx
+++ b/watchlists/exceptions.xlsx
@@ -1,23 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exceptions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Exceptions" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="3">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="dd/mmm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,22 +28,55 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="FF808080"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="0"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <i val="1"/>
+      <color rgb="FF808080"/>
+      <sz val="11"/>
+    </font>
+    <font>
       <b val="1"/>
     </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00808080"/>
-    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -49,18 +84,84 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9E1F2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9E1F2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9E1F2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9E1F2"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="5">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF70AD47"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -422,92 +523,427 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="21" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="4"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Symbol</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Date From</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Date To</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>Reason</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Date From</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Date To</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>EXAMPLE1</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Too volatile - remove this row and add your own</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>HSHP</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="n">
+        <v>46226</v>
+      </c>
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>31/Sept/2026</t>
+        </is>
+      </c>
+      <c r="D2" s="11" t="inlineStr">
+        <is>
+          <t>Bought this stocks</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>EXAMPLE2</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Under regulatory review - replace with real tickers</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>01/Jan/2026</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>31/Dec/2026</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>TRGP</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="n">
+        <v>46227</v>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>31/Sept/2026</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>Bought this stocks</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>EXAMPLE3</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Already holding this position - customize as needed</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>01/Jun/2026</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr"/>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>SB</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="n">
+        <v>46227</v>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>31/Sept/2026</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Bought this stocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>SOBO</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="n">
+        <v>46226</v>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>31/Sept/2026</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Bought this stocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>FTI</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>46226</v>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>31/Sept/2026</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Bought this stocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>EC</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>46227</v>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>31/Sept/2026</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Bought this stocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>KNTK</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>46227</v>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>31/Sept/2026</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Bought this stocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>GNK</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>46226</v>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>31/Sept/2026</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Bought this stocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>ADM</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>46226</v>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>31/Sept/2026</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Bought this stocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>PBA</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>46227</v>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>31/Sept/2026</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Bought this stocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>WAB</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>46226</v>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>31/Sept/2026</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Bought this stocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>46227</v>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>31/Sept/2026</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>Bought this stocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>TRP</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="n">
+        <v>46226</v>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>31/Sept/2026</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Bought this stocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>HESM</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="n">
+        <v>46226</v>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>31/Sept/2026</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Bought this stocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>ADX</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="n">
+        <v>46226</v>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>31/Sept/2026</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Bought this stocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>FTS</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="n">
+        <v>46226</v>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>31/Sept/2026</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>Bought this stocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="n">
+        <v>46226</v>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>31/Sept/2026</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>Bought this stocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>TDY</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="n">
+        <v>46226</v>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>31/Sept/2026</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>Bought this stocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="C20" s="12" t="n"/>
+      <c r="D20" s="12" t="n"/>
+    </row>
+    <row r="21">
+      <c r="C21" s="12" t="n"/>
+      <c r="D21" s="12" t="n"/>
+    </row>
+    <row r="22">
+      <c r="C22" s="12" t="n"/>
+      <c r="D22" s="12" t="n"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A2:A19">
+    <cfRule type="expression" priority="1" dxfId="4">
+      <formula>ISNUMBER(SEARCH("STRONG BUY",$Q2))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="3">
+      <formula>AND(ISNUMBER(SEARCH("BUY",$Q2)),NOT(ISNUMBER(SEARCH("STRONG BUY",$Q2))))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="2">
+      <formula>OR(ISNUMBER(SEARCH("ACCUMULATE",$Q2)),ISNUMBER(SEARCH("HOLD",$Q2)))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="1">
+      <formula>ISNUMBER(SEARCH("WATCH",$Q2))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="0">
+      <formula>ISNUMBER(SEARCH("AVOID",$Q2))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>